<commit_message>
Update NCAA bracket and regenerate TS data files
Bradley in at South-14, Yale at East-12, High Point at West-12,
SF Austin at South-12, Liberty at Midwest-13. IL Chicago removed.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ProjectedBrackets.xlsx
+++ b/ProjectedBrackets.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e9f237e831f26750/Jupyter/Business/MM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="260" documentId="8_{DC458501-F46D-487D-A95A-F0D26D9143CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5463424-5DB8-40AA-8FB8-33587EA271BF}"/>
+  <xr:revisionPtr revIDLastSave="267" documentId="8_{DC458501-F46D-487D-A95A-F0D26D9143CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7DF59166-924F-46DC-80D5-AB780EF9B925}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{6E9E6780-D9B8-4788-9082-4844BD7B8591}"/>
   </bookViews>
@@ -1309,7 +1309,7 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>147</v>
+        <v>33</v>
       </c>
       <c r="B14" t="s">
         <v>4</v>
@@ -1496,7 +1496,7 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>71</v>
+        <v>53</v>
       </c>
       <c r="B31" t="s">
         <v>37</v>
@@ -1507,7 +1507,7 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>183</v>
+        <v>35</v>
       </c>
       <c r="B32" t="s">
         <v>37</v>
@@ -1518,7 +1518,7 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>35</v>
+        <v>144</v>
       </c>
       <c r="B33" t="s">
         <v>37</v>
@@ -1694,7 +1694,7 @@
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="B49" t="s">
         <v>58</v>
@@ -1870,7 +1870,7 @@
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>33</v>
+        <v>88</v>
       </c>
       <c r="B65" t="s">
         <v>76</v>
@@ -1881,7 +1881,7 @@
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>53</v>
+        <v>183</v>
       </c>
       <c r="B66" t="s">
         <v>76</v>

</xml_diff>